<commit_message>
Rebuild forecast with literal cadence (4 = every 4 weeks)
- Correct 4-weekly payers (Birmingham, Walsall SL, etc.) to land once
  every 28 days instead of every week; freq 2 fortnightly, freq 1 weekly,
  HB rows daily GBP4000
- Anchor each payer to its last May payment and step forward
- Rebuild June 2026 -> March 2027; monthly totals now ~GBP1.7-1.9M,
  consistent with reconciled actuals
- Update working note

https://claude.ai/code/session_01V6KrsFLkztukGdQb6oLmYN
</commit_message>
<xml_diff>
--- a/Income_forecast_2026.xlsx
+++ b/Income_forecast_2026.xlsx
@@ -1595,18 +1595,12 @@
           <t>Birmingham City Council - Supported Living</t>
         </is>
       </c>
-      <c r="F3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
+      <c r="F3" s="11" t="n"/>
       <c r="M3" s="11" t="n">
         <v>59419.08</v>
       </c>
-      <c r="T3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
-      <c r="AA3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
+      <c r="T3" s="11" t="n"/>
+      <c r="AA3" s="11" t="n"/>
       <c r="AF3" s="12">
         <f>SUM(B3:AE3)</f>
         <v/>
@@ -1635,6 +1629,9 @@
       <c r="Q5" s="11" t="n">
         <v>41250.75</v>
       </c>
+      <c r="AE5" s="11" t="n">
+        <v>41250.75</v>
+      </c>
       <c r="AF5" s="12">
         <f>SUM(B5:AE5)</f>
         <v/>
@@ -1646,10 +1643,12 @@
           <t>Sandwell MBC - Daycare</t>
         </is>
       </c>
-      <c r="G6" s="11" t="n">
+      <c r="G6" s="11" t="n"/>
+      <c r="N6" s="11" t="n">
         <v>6585.35</v>
       </c>
-      <c r="U6" s="11" t="n">
+      <c r="U6" s="11" t="n"/>
+      <c r="AB6" s="11" t="n">
         <v>6585.35</v>
       </c>
       <c r="AF6" s="12">
@@ -1697,18 +1696,12 @@
           <t>Walsall - Respite</t>
         </is>
       </c>
-      <c r="D9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
+      <c r="D9" s="11" t="n"/>
       <c r="K9" s="11" t="n">
         <v>11460.8</v>
       </c>
-      <c r="R9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
-      <c r="Y9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
+      <c r="R9" s="11" t="n"/>
+      <c r="Y9" s="11" t="n"/>
       <c r="AF9" s="12">
         <f>SUM(B9:AE9)</f>
         <v/>
@@ -1731,18 +1724,12 @@
           <t>Ideal for All Ltd - Direct Payments</t>
         </is>
       </c>
-      <c r="G11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
+      <c r="G11" s="11" t="n"/>
       <c r="N11" s="11" t="n">
         <v>4131.62</v>
       </c>
-      <c r="U11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
-      <c r="AB11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
+      <c r="U11" s="11" t="n"/>
+      <c r="AB11" s="11" t="n"/>
       <c r="AF11" s="12">
         <f>SUM(B11:AE11)</f>
         <v/>
@@ -1754,18 +1741,12 @@
           <t>Kirklees - Supported Living</t>
         </is>
       </c>
-      <c r="D12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
+      <c r="D12" s="11" t="n"/>
       <c r="K12" s="11" t="n">
         <v>5458.48</v>
       </c>
-      <c r="R12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
-      <c r="Y12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
+      <c r="R12" s="11" t="n"/>
+      <c r="Y12" s="11" t="n"/>
       <c r="AF12" s="12">
         <f>SUM(B12:AE12)</f>
         <v/>
@@ -1777,18 +1758,12 @@
           <t>LB Hillingdon - Supported Living</t>
         </is>
       </c>
-      <c r="E13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
+      <c r="E13" s="11" t="n"/>
       <c r="L13" s="11" t="n">
         <v>5203.8</v>
       </c>
-      <c r="S13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
-      <c r="Z13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
+      <c r="S13" s="11" t="n"/>
+      <c r="Z13" s="11" t="n"/>
       <c r="AF13" s="12">
         <f>SUM(B13:AE13)</f>
         <v/>
@@ -1800,18 +1775,12 @@
           <t>NHS Birmingham &amp; Solihull ICB</t>
         </is>
       </c>
-      <c r="F14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
+      <c r="F14" s="11" t="n"/>
       <c r="M14" s="11" t="n">
         <v>7814.17</v>
       </c>
-      <c r="T14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
-      <c r="AA14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
+      <c r="T14" s="11" t="n"/>
+      <c r="AA14" s="11" t="n"/>
       <c r="AF14" s="12">
         <f>SUM(B14:AE14)</f>
         <v/>
@@ -1823,18 +1792,12 @@
           <t>NHS Black Country ICB</t>
         </is>
       </c>
-      <c r="F15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
+      <c r="F15" s="11" t="n"/>
       <c r="M15" s="11" t="n">
         <v>5499.45</v>
       </c>
-      <c r="T15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
-      <c r="AA15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
+      <c r="T15" s="11" t="n"/>
+      <c r="AA15" s="11" t="n"/>
       <c r="AF15" s="12">
         <f>SUM(B15:AE15)</f>
         <v/>
@@ -1947,7 +1910,8 @@
           <t>Sandwell MBC - Supported Living</t>
         </is>
       </c>
-      <c r="C17" s="11" t="n">
+      <c r="C17" s="11" t="n"/>
+      <c r="J17" s="11" t="n">
         <v>132834.8</v>
       </c>
       <c r="X17" s="11" t="n">
@@ -1964,21 +1928,13 @@
           <t>Solihull MBC - Supported Living</t>
         </is>
       </c>
-      <c r="B18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
-      <c r="I18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
+      <c r="B18" s="11" t="n"/>
+      <c r="I18" s="11" t="n"/>
       <c r="P18" s="11" t="n">
         <v>33031.6</v>
       </c>
-      <c r="W18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
-      <c r="AD18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
+      <c r="W18" s="11" t="n"/>
+      <c r="AD18" s="11" t="n"/>
       <c r="AF18" s="12">
         <f>SUM(B18:AE18)</f>
         <v/>
@@ -1990,18 +1946,12 @@
           <t>Walsall - Supported Living</t>
         </is>
       </c>
-      <c r="D19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
+      <c r="D19" s="11" t="n"/>
       <c r="K19" s="11" t="n">
         <v>319655.76</v>
       </c>
-      <c r="R19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
-      <c r="Y19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
+      <c r="R19" s="11" t="n"/>
+      <c r="Y19" s="11" t="n"/>
       <c r="AF19" s="12">
         <f>SUM(B19:AE19)</f>
         <v/>
@@ -2036,18 +1986,12 @@
           <t>People Plus - Direct Payments</t>
         </is>
       </c>
-      <c r="F21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
+      <c r="F21" s="11" t="n"/>
       <c r="M21" s="11" t="n">
         <v>21527.2</v>
       </c>
-      <c r="T21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
-      <c r="AA21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
+      <c r="T21" s="11" t="n"/>
+      <c r="AA21" s="11" t="n"/>
       <c r="AF21" s="12">
         <f>SUM(B21:AE21)</f>
         <v/>
@@ -2059,18 +2003,12 @@
           <t>Middlesbrough - Supported Living</t>
         </is>
       </c>
-      <c r="F22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
+      <c r="F22" s="11" t="n"/>
       <c r="M22" s="11" t="n">
         <v>6115.4</v>
       </c>
-      <c r="T22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
-      <c r="AA22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
+      <c r="T22" s="11" t="n"/>
+      <c r="AA22" s="11" t="n"/>
       <c r="AF22" s="12">
         <f>SUM(B22:AE22)</f>
         <v/>
@@ -2735,21 +2673,13 @@
           <t>Birmingham City Council - Supported Living</t>
         </is>
       </c>
-      <c r="D3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
+      <c r="D3" s="11" t="n"/>
       <c r="K3" s="11" t="n">
         <v>59419.08</v>
       </c>
-      <c r="R3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
-      <c r="Y3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
-      <c r="AF3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
+      <c r="R3" s="11" t="n"/>
+      <c r="Y3" s="11" t="n"/>
+      <c r="AF3" s="11" t="n"/>
       <c r="AG3" s="12">
         <f>SUM(B3:AF3)</f>
         <v/>
@@ -2772,10 +2702,12 @@
           <t>Sandwell MBC - Respite</t>
         </is>
       </c>
-      <c r="H5" s="11" t="n">
+      <c r="H5" s="11" t="n"/>
+      <c r="O5" s="11" t="n">
         <v>41250.75</v>
       </c>
-      <c r="V5" s="11" t="n">
+      <c r="V5" s="11" t="n"/>
+      <c r="AC5" s="11" t="n">
         <v>41250.75</v>
       </c>
       <c r="AG5" s="12">
@@ -2789,10 +2721,12 @@
           <t>Sandwell MBC - Daycare</t>
         </is>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="E6" s="11" t="n"/>
+      <c r="L6" s="11" t="n">
         <v>6585.35</v>
       </c>
-      <c r="S6" s="11" t="n">
+      <c r="S6" s="11" t="n"/>
+      <c r="Z6" s="11" t="n">
         <v>6585.35</v>
       </c>
       <c r="AG6" s="12">
@@ -2843,21 +2777,13 @@
           <t>Walsall - Respite</t>
         </is>
       </c>
-      <c r="B9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
+      <c r="B9" s="11" t="n"/>
       <c r="I9" s="11" t="n">
         <v>11460.8</v>
       </c>
-      <c r="P9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
-      <c r="W9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
-      <c r="AD9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
+      <c r="P9" s="11" t="n"/>
+      <c r="W9" s="11" t="n"/>
+      <c r="AD9" s="11" t="n"/>
       <c r="AG9" s="12">
         <f>SUM(B9:AF9)</f>
         <v/>
@@ -2880,18 +2806,12 @@
           <t>Ideal for All Ltd - Direct Payments</t>
         </is>
       </c>
-      <c r="E11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
+      <c r="E11" s="11" t="n"/>
       <c r="L11" s="11" t="n">
         <v>4131.62</v>
       </c>
-      <c r="S11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
-      <c r="Z11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
+      <c r="S11" s="11" t="n"/>
+      <c r="Z11" s="11" t="n"/>
       <c r="AG11" s="12">
         <f>SUM(B11:AF11)</f>
         <v/>
@@ -2903,21 +2823,13 @@
           <t>Kirklees - Supported Living</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
+      <c r="B12" s="11" t="n"/>
       <c r="I12" s="11" t="n">
         <v>5458.48</v>
       </c>
-      <c r="P12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
-      <c r="W12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
-      <c r="AD12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
+      <c r="P12" s="11" t="n"/>
+      <c r="W12" s="11" t="n"/>
+      <c r="AD12" s="11" t="n"/>
       <c r="AG12" s="12">
         <f>SUM(B12:AF12)</f>
         <v/>
@@ -2929,21 +2841,13 @@
           <t>LB Hillingdon - Supported Living</t>
         </is>
       </c>
-      <c r="C13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
+      <c r="C13" s="11" t="n"/>
       <c r="J13" s="11" t="n">
         <v>5203.8</v>
       </c>
-      <c r="Q13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
-      <c r="X13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
-      <c r="AE13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
+      <c r="Q13" s="11" t="n"/>
+      <c r="X13" s="11" t="n"/>
+      <c r="AE13" s="11" t="n"/>
       <c r="AG13" s="12">
         <f>SUM(B13:AF13)</f>
         <v/>
@@ -2955,21 +2859,13 @@
           <t>NHS Birmingham &amp; Solihull ICB</t>
         </is>
       </c>
-      <c r="D14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
+      <c r="D14" s="11" t="n"/>
       <c r="K14" s="11" t="n">
         <v>7814.17</v>
       </c>
-      <c r="R14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
-      <c r="Y14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
-      <c r="AF14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
+      <c r="R14" s="11" t="n"/>
+      <c r="Y14" s="11" t="n"/>
+      <c r="AF14" s="11" t="n"/>
       <c r="AG14" s="12">
         <f>SUM(B14:AF14)</f>
         <v/>
@@ -2981,21 +2877,13 @@
           <t>NHS Black Country ICB</t>
         </is>
       </c>
-      <c r="D15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
+      <c r="D15" s="11" t="n"/>
       <c r="K15" s="11" t="n">
         <v>5499.45</v>
       </c>
-      <c r="R15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
-      <c r="Y15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
-      <c r="AF15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
+      <c r="R15" s="11" t="n"/>
+      <c r="Y15" s="11" t="n"/>
+      <c r="AF15" s="11" t="n"/>
       <c r="AG15" s="12">
         <f>SUM(B15:AF15)</f>
         <v/>
@@ -3114,9 +3002,10 @@
       <c r="H17" s="11" t="n">
         <v>132834.8</v>
       </c>
-      <c r="AC17" s="11" t="n">
+      <c r="V17" s="11" t="n">
         <v>132834.8</v>
       </c>
+      <c r="AC17" s="11" t="n"/>
       <c r="AG17" s="12">
         <f>SUM(B17:AF17)</f>
         <v/>
@@ -3128,18 +3017,12 @@
           <t>Solihull MBC - Supported Living</t>
         </is>
       </c>
-      <c r="G18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
+      <c r="G18" s="11" t="n"/>
       <c r="N18" s="11" t="n">
         <v>33031.6</v>
       </c>
-      <c r="U18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
-      <c r="AB18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
+      <c r="U18" s="11" t="n"/>
+      <c r="AB18" s="11" t="n"/>
       <c r="AG18" s="12">
         <f>SUM(B18:AF18)</f>
         <v/>
@@ -3151,21 +3034,13 @@
           <t>Walsall - Supported Living</t>
         </is>
       </c>
-      <c r="B19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
+      <c r="B19" s="11" t="n"/>
       <c r="I19" s="11" t="n">
         <v>319655.76</v>
       </c>
-      <c r="P19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
-      <c r="W19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
-      <c r="AD19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
+      <c r="P19" s="11" t="n"/>
+      <c r="W19" s="11" t="n"/>
+      <c r="AD19" s="11" t="n"/>
       <c r="AG19" s="12">
         <f>SUM(B19:AF19)</f>
         <v/>
@@ -3203,21 +3078,13 @@
           <t>People Plus - Direct Payments</t>
         </is>
       </c>
-      <c r="D21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
+      <c r="D21" s="11" t="n"/>
       <c r="K21" s="11" t="n">
         <v>21527.2</v>
       </c>
-      <c r="R21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
-      <c r="Y21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
-      <c r="AF21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
+      <c r="R21" s="11" t="n"/>
+      <c r="Y21" s="11" t="n"/>
+      <c r="AF21" s="11" t="n"/>
       <c r="AG21" s="12">
         <f>SUM(B21:AF21)</f>
         <v/>
@@ -3229,21 +3096,13 @@
           <t>Middlesbrough - Supported Living</t>
         </is>
       </c>
-      <c r="D22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
+      <c r="D22" s="11" t="n"/>
       <c r="K22" s="11" t="n">
         <v>6115.4</v>
       </c>
-      <c r="R22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
-      <c r="Y22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
-      <c r="AF22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
+      <c r="R22" s="11" t="n"/>
+      <c r="Y22" s="11" t="n"/>
+      <c r="AF22" s="11" t="n"/>
       <c r="AG22" s="12">
         <f>SUM(B22:AF22)</f>
         <v/>
@@ -3933,27 +3792,21 @@
       <c r="L3" s="11" t="n"/>
       <c r="M3" s="11" t="n"/>
       <c r="N3" s="11" t="n"/>
-      <c r="O3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
+      <c r="O3" s="11" t="n"/>
       <c r="P3" s="11" t="n"/>
       <c r="Q3" s="11" t="n"/>
       <c r="R3" s="11" t="n"/>
       <c r="S3" s="11" t="n"/>
       <c r="T3" s="11" t="n"/>
       <c r="U3" s="11" t="n"/>
-      <c r="V3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
+      <c r="V3" s="11" t="n"/>
       <c r="W3" s="11" t="n"/>
       <c r="X3" s="11" t="n"/>
       <c r="Y3" s="11" t="n"/>
       <c r="Z3" s="11" t="n"/>
       <c r="AA3" s="11" t="n"/>
       <c r="AB3" s="11" t="n"/>
-      <c r="AC3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
+      <c r="AC3" s="11" t="n"/>
       <c r="AD3" s="11" t="n"/>
       <c r="AE3" s="11" t="n"/>
       <c r="AF3" s="11" t="n"/>
@@ -4013,32 +3866,32 @@
       <c r="B5" s="11" t="n"/>
       <c r="C5" s="11" t="n"/>
       <c r="D5" s="11" t="n"/>
-      <c r="E5" s="11" t="n">
-        <v>41250.75</v>
-      </c>
+      <c r="E5" s="11" t="n"/>
       <c r="F5" s="11" t="n"/>
       <c r="G5" s="11" t="n"/>
       <c r="H5" s="11" t="n"/>
       <c r="I5" s="11" t="n"/>
       <c r="J5" s="11" t="n"/>
       <c r="K5" s="11" t="n"/>
-      <c r="L5" s="11" t="n"/>
+      <c r="L5" s="11" t="n">
+        <v>41250.75</v>
+      </c>
       <c r="M5" s="11" t="n"/>
       <c r="N5" s="11" t="n"/>
       <c r="O5" s="11" t="n"/>
       <c r="P5" s="11" t="n"/>
       <c r="Q5" s="11" t="n"/>
       <c r="R5" s="11" t="n"/>
-      <c r="S5" s="11" t="n">
-        <v>41250.75</v>
-      </c>
+      <c r="S5" s="11" t="n"/>
       <c r="T5" s="11" t="n"/>
       <c r="U5" s="11" t="n"/>
       <c r="V5" s="11" t="n"/>
       <c r="W5" s="11" t="n"/>
       <c r="X5" s="11" t="n"/>
       <c r="Y5" s="11" t="n"/>
-      <c r="Z5" s="11" t="n"/>
+      <c r="Z5" s="11" t="n">
+        <v>41250.75</v>
+      </c>
       <c r="AA5" s="11" t="n"/>
       <c r="AB5" s="11" t="n"/>
       <c r="AC5" s="11" t="n"/>
@@ -4056,32 +3909,32 @@
           <t>Sandwell MBC - Daycare</t>
         </is>
       </c>
-      <c r="B6" s="11" t="n">
-        <v>6585.35</v>
-      </c>
+      <c r="B6" s="11" t="n"/>
       <c r="C6" s="11" t="n"/>
       <c r="D6" s="11" t="n"/>
       <c r="E6" s="11" t="n"/>
       <c r="F6" s="11" t="n"/>
       <c r="G6" s="11" t="n"/>
       <c r="H6" s="11" t="n"/>
-      <c r="I6" s="11" t="n"/>
+      <c r="I6" s="11" t="n">
+        <v>6585.35</v>
+      </c>
       <c r="J6" s="11" t="n"/>
       <c r="K6" s="11" t="n"/>
       <c r="L6" s="11" t="n"/>
       <c r="M6" s="11" t="n"/>
       <c r="N6" s="11" t="n"/>
       <c r="O6" s="11" t="n"/>
-      <c r="P6" s="11" t="n">
-        <v>6585.35</v>
-      </c>
+      <c r="P6" s="11" t="n"/>
       <c r="Q6" s="11" t="n"/>
       <c r="R6" s="11" t="n"/>
       <c r="S6" s="11" t="n"/>
       <c r="T6" s="11" t="n"/>
       <c r="U6" s="11" t="n"/>
       <c r="V6" s="11" t="n"/>
-      <c r="W6" s="11" t="n"/>
+      <c r="W6" s="11" t="n">
+        <v>6585.35</v>
+      </c>
       <c r="X6" s="11" t="n"/>
       <c r="Y6" s="11" t="n"/>
       <c r="Z6" s="11" t="n"/>
@@ -4207,27 +4060,21 @@
       <c r="J9" s="11" t="n"/>
       <c r="K9" s="11" t="n"/>
       <c r="L9" s="11" t="n"/>
-      <c r="M9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
+      <c r="M9" s="11" t="n"/>
       <c r="N9" s="11" t="n"/>
       <c r="O9" s="11" t="n"/>
       <c r="P9" s="11" t="n"/>
       <c r="Q9" s="11" t="n"/>
       <c r="R9" s="11" t="n"/>
       <c r="S9" s="11" t="n"/>
-      <c r="T9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
+      <c r="T9" s="11" t="n"/>
       <c r="U9" s="11" t="n"/>
       <c r="V9" s="11" t="n"/>
       <c r="W9" s="11" t="n"/>
       <c r="X9" s="11" t="n"/>
       <c r="Y9" s="11" t="n"/>
       <c r="Z9" s="11" t="n"/>
-      <c r="AA9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
+      <c r="AA9" s="11" t="n"/>
       <c r="AB9" s="11" t="n"/>
       <c r="AC9" s="11" t="n"/>
       <c r="AD9" s="11" t="n"/>
@@ -4286,9 +4133,7 @@
           <t>Ideal for All Ltd - Direct Payments</t>
         </is>
       </c>
-      <c r="B11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
+      <c r="B11" s="11" t="n"/>
       <c r="C11" s="11" t="n"/>
       <c r="D11" s="11" t="n"/>
       <c r="E11" s="11" t="n"/>
@@ -4304,27 +4149,21 @@
       <c r="M11" s="11" t="n"/>
       <c r="N11" s="11" t="n"/>
       <c r="O11" s="11" t="n"/>
-      <c r="P11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
+      <c r="P11" s="11" t="n"/>
       <c r="Q11" s="11" t="n"/>
       <c r="R11" s="11" t="n"/>
       <c r="S11" s="11" t="n"/>
       <c r="T11" s="11" t="n"/>
       <c r="U11" s="11" t="n"/>
       <c r="V11" s="11" t="n"/>
-      <c r="W11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
+      <c r="W11" s="11" t="n"/>
       <c r="X11" s="11" t="n"/>
       <c r="Y11" s="11" t="n"/>
       <c r="Z11" s="11" t="n"/>
       <c r="AA11" s="11" t="n"/>
       <c r="AB11" s="11" t="n"/>
       <c r="AC11" s="11" t="n"/>
-      <c r="AD11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
+      <c r="AD11" s="11" t="n"/>
       <c r="AE11" s="11" t="n"/>
       <c r="AF11" s="11" t="n"/>
       <c r="AG11" s="12">
@@ -4351,27 +4190,21 @@
       <c r="J12" s="11" t="n"/>
       <c r="K12" s="11" t="n"/>
       <c r="L12" s="11" t="n"/>
-      <c r="M12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
+      <c r="M12" s="11" t="n"/>
       <c r="N12" s="11" t="n"/>
       <c r="O12" s="11" t="n"/>
       <c r="P12" s="11" t="n"/>
       <c r="Q12" s="11" t="n"/>
       <c r="R12" s="11" t="n"/>
       <c r="S12" s="11" t="n"/>
-      <c r="T12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
+      <c r="T12" s="11" t="n"/>
       <c r="U12" s="11" t="n"/>
       <c r="V12" s="11" t="n"/>
       <c r="W12" s="11" t="n"/>
       <c r="X12" s="11" t="n"/>
       <c r="Y12" s="11" t="n"/>
       <c r="Z12" s="11" t="n"/>
-      <c r="AA12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
+      <c r="AA12" s="11" t="n"/>
       <c r="AB12" s="11" t="n"/>
       <c r="AC12" s="11" t="n"/>
       <c r="AD12" s="11" t="n"/>
@@ -4402,27 +4235,21 @@
       <c r="K13" s="11" t="n"/>
       <c r="L13" s="11" t="n"/>
       <c r="M13" s="11" t="n"/>
-      <c r="N13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
+      <c r="N13" s="11" t="n"/>
       <c r="O13" s="11" t="n"/>
       <c r="P13" s="11" t="n"/>
       <c r="Q13" s="11" t="n"/>
       <c r="R13" s="11" t="n"/>
       <c r="S13" s="11" t="n"/>
       <c r="T13" s="11" t="n"/>
-      <c r="U13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
+      <c r="U13" s="11" t="n"/>
       <c r="V13" s="11" t="n"/>
       <c r="W13" s="11" t="n"/>
       <c r="X13" s="11" t="n"/>
       <c r="Y13" s="11" t="n"/>
       <c r="Z13" s="11" t="n"/>
       <c r="AA13" s="11" t="n"/>
-      <c r="AB13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
+      <c r="AB13" s="11" t="n"/>
       <c r="AC13" s="11" t="n"/>
       <c r="AD13" s="11" t="n"/>
       <c r="AE13" s="11" t="n"/>
@@ -4453,27 +4280,21 @@
       <c r="L14" s="11" t="n"/>
       <c r="M14" s="11" t="n"/>
       <c r="N14" s="11" t="n"/>
-      <c r="O14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
+      <c r="O14" s="11" t="n"/>
       <c r="P14" s="11" t="n"/>
       <c r="Q14" s="11" t="n"/>
       <c r="R14" s="11" t="n"/>
       <c r="S14" s="11" t="n"/>
       <c r="T14" s="11" t="n"/>
       <c r="U14" s="11" t="n"/>
-      <c r="V14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
+      <c r="V14" s="11" t="n"/>
       <c r="W14" s="11" t="n"/>
       <c r="X14" s="11" t="n"/>
       <c r="Y14" s="11" t="n"/>
       <c r="Z14" s="11" t="n"/>
       <c r="AA14" s="11" t="n"/>
       <c r="AB14" s="11" t="n"/>
-      <c r="AC14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
+      <c r="AC14" s="11" t="n"/>
       <c r="AD14" s="11" t="n"/>
       <c r="AE14" s="11" t="n"/>
       <c r="AF14" s="11" t="n"/>
@@ -4503,27 +4324,21 @@
       <c r="L15" s="11" t="n"/>
       <c r="M15" s="11" t="n"/>
       <c r="N15" s="11" t="n"/>
-      <c r="O15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
+      <c r="O15" s="11" t="n"/>
       <c r="P15" s="11" t="n"/>
       <c r="Q15" s="11" t="n"/>
       <c r="R15" s="11" t="n"/>
       <c r="S15" s="11" t="n"/>
       <c r="T15" s="11" t="n"/>
       <c r="U15" s="11" t="n"/>
-      <c r="V15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
+      <c r="V15" s="11" t="n"/>
       <c r="W15" s="11" t="n"/>
       <c r="X15" s="11" t="n"/>
       <c r="Y15" s="11" t="n"/>
       <c r="Z15" s="11" t="n"/>
       <c r="AA15" s="11" t="n"/>
       <c r="AB15" s="11" t="n"/>
-      <c r="AC15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
+      <c r="AC15" s="11" t="n"/>
       <c r="AD15" s="11" t="n"/>
       <c r="AE15" s="11" t="n"/>
       <c r="AF15" s="11" t="n"/>
@@ -4661,16 +4476,16 @@
       <c r="P17" s="11" t="n"/>
       <c r="Q17" s="11" t="n"/>
       <c r="R17" s="11" t="n"/>
-      <c r="S17" s="11" t="n"/>
+      <c r="S17" s="11" t="n">
+        <v>132834.8</v>
+      </c>
       <c r="T17" s="11" t="n"/>
       <c r="U17" s="11" t="n"/>
       <c r="V17" s="11" t="n"/>
       <c r="W17" s="11" t="n"/>
       <c r="X17" s="11" t="n"/>
       <c r="Y17" s="11" t="n"/>
-      <c r="Z17" s="11" t="n">
-        <v>132834.8</v>
-      </c>
+      <c r="Z17" s="11" t="n"/>
       <c r="AA17" s="11" t="n"/>
       <c r="AB17" s="11" t="n"/>
       <c r="AC17" s="11" t="n"/>
@@ -4690,9 +4505,7 @@
       </c>
       <c r="B18" s="11" t="n"/>
       <c r="C18" s="11" t="n"/>
-      <c r="D18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
+      <c r="D18" s="11" t="n"/>
       <c r="E18" s="11" t="n"/>
       <c r="F18" s="11" t="n"/>
       <c r="G18" s="11" t="n"/>
@@ -4708,27 +4521,21 @@
       <c r="O18" s="11" t="n"/>
       <c r="P18" s="11" t="n"/>
       <c r="Q18" s="11" t="n"/>
-      <c r="R18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
+      <c r="R18" s="11" t="n"/>
       <c r="S18" s="11" t="n"/>
       <c r="T18" s="11" t="n"/>
       <c r="U18" s="11" t="n"/>
       <c r="V18" s="11" t="n"/>
       <c r="W18" s="11" t="n"/>
       <c r="X18" s="11" t="n"/>
-      <c r="Y18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
+      <c r="Y18" s="11" t="n"/>
       <c r="Z18" s="11" t="n"/>
       <c r="AA18" s="11" t="n"/>
       <c r="AB18" s="11" t="n"/>
       <c r="AC18" s="11" t="n"/>
       <c r="AD18" s="11" t="n"/>
       <c r="AE18" s="11" t="n"/>
-      <c r="AF18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
+      <c r="AF18" s="11" t="n"/>
       <c r="AG18" s="12">
         <f>SUM(B18:AF18)</f>
         <v/>
@@ -4753,27 +4560,21 @@
       <c r="J19" s="11" t="n"/>
       <c r="K19" s="11" t="n"/>
       <c r="L19" s="11" t="n"/>
-      <c r="M19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
+      <c r="M19" s="11" t="n"/>
       <c r="N19" s="11" t="n"/>
       <c r="O19" s="11" t="n"/>
       <c r="P19" s="11" t="n"/>
       <c r="Q19" s="11" t="n"/>
       <c r="R19" s="11" t="n"/>
       <c r="S19" s="11" t="n"/>
-      <c r="T19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
+      <c r="T19" s="11" t="n"/>
       <c r="U19" s="11" t="n"/>
       <c r="V19" s="11" t="n"/>
       <c r="W19" s="11" t="n"/>
       <c r="X19" s="11" t="n"/>
       <c r="Y19" s="11" t="n"/>
       <c r="Z19" s="11" t="n"/>
-      <c r="AA19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
+      <c r="AA19" s="11" t="n"/>
       <c r="AB19" s="11" t="n"/>
       <c r="AC19" s="11" t="n"/>
       <c r="AD19" s="11" t="n"/>
@@ -4855,27 +4656,21 @@
       <c r="L21" s="11" t="n"/>
       <c r="M21" s="11" t="n"/>
       <c r="N21" s="11" t="n"/>
-      <c r="O21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
+      <c r="O21" s="11" t="n"/>
       <c r="P21" s="11" t="n"/>
       <c r="Q21" s="11" t="n"/>
       <c r="R21" s="11" t="n"/>
       <c r="S21" s="11" t="n"/>
       <c r="T21" s="11" t="n"/>
       <c r="U21" s="11" t="n"/>
-      <c r="V21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
+      <c r="V21" s="11" t="n"/>
       <c r="W21" s="11" t="n"/>
       <c r="X21" s="11" t="n"/>
       <c r="Y21" s="11" t="n"/>
       <c r="Z21" s="11" t="n"/>
       <c r="AA21" s="11" t="n"/>
       <c r="AB21" s="11" t="n"/>
-      <c r="AC21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
+      <c r="AC21" s="11" t="n"/>
       <c r="AD21" s="11" t="n"/>
       <c r="AE21" s="11" t="n"/>
       <c r="AF21" s="11" t="n"/>
@@ -4905,27 +4700,21 @@
       <c r="L22" s="11" t="n"/>
       <c r="M22" s="11" t="n"/>
       <c r="N22" s="11" t="n"/>
-      <c r="O22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
+      <c r="O22" s="11" t="n"/>
       <c r="P22" s="11" t="n"/>
       <c r="Q22" s="11" t="n"/>
       <c r="R22" s="11" t="n"/>
       <c r="S22" s="11" t="n"/>
       <c r="T22" s="11" t="n"/>
       <c r="U22" s="11" t="n"/>
-      <c r="V22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
+      <c r="V22" s="11" t="n"/>
       <c r="W22" s="11" t="n"/>
       <c r="X22" s="11" t="n"/>
       <c r="Y22" s="11" t="n"/>
       <c r="Z22" s="11" t="n"/>
       <c r="AA22" s="11" t="n"/>
       <c r="AB22" s="11" t="n"/>
-      <c r="AC22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
+      <c r="AC22" s="11" t="n"/>
       <c r="AD22" s="11" t="n"/>
       <c r="AE22" s="11" t="n"/>
       <c r="AF22" s="11" t="n"/>
@@ -5618,27 +5407,21 @@
       <c r="I3" s="11" t="n"/>
       <c r="J3" s="11" t="n"/>
       <c r="K3" s="11" t="n"/>
-      <c r="L3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
+      <c r="L3" s="11" t="n"/>
       <c r="M3" s="11" t="n"/>
       <c r="N3" s="11" t="n"/>
       <c r="O3" s="11" t="n"/>
       <c r="P3" s="11" t="n"/>
       <c r="Q3" s="11" t="n"/>
       <c r="R3" s="11" t="n"/>
-      <c r="S3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
+      <c r="S3" s="11" t="n"/>
       <c r="T3" s="11" t="n"/>
       <c r="U3" s="11" t="n"/>
       <c r="V3" s="11" t="n"/>
       <c r="W3" s="11" t="n"/>
       <c r="X3" s="11" t="n"/>
       <c r="Y3" s="11" t="n"/>
-      <c r="Z3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
+      <c r="Z3" s="11" t="n"/>
       <c r="AA3" s="11" t="n"/>
       <c r="AB3" s="11" t="n"/>
       <c r="AC3" s="11" t="n"/>
@@ -5692,32 +5475,32 @@
           <t>Sandwell MBC - Respite</t>
         </is>
       </c>
-      <c r="B5" s="11" t="n">
-        <v>41250.75</v>
-      </c>
+      <c r="B5" s="11" t="n"/>
       <c r="C5" s="11" t="n"/>
       <c r="D5" s="11" t="n"/>
       <c r="E5" s="11" t="n"/>
       <c r="F5" s="11" t="n"/>
       <c r="G5" s="11" t="n"/>
       <c r="H5" s="11" t="n"/>
-      <c r="I5" s="11" t="n"/>
+      <c r="I5" s="11" t="n">
+        <v>41250.75</v>
+      </c>
       <c r="J5" s="11" t="n"/>
       <c r="K5" s="11" t="n"/>
       <c r="L5" s="11" t="n"/>
       <c r="M5" s="11" t="n"/>
       <c r="N5" s="11" t="n"/>
       <c r="O5" s="11" t="n"/>
-      <c r="P5" s="11" t="n">
-        <v>41250.75</v>
-      </c>
+      <c r="P5" s="11" t="n"/>
       <c r="Q5" s="11" t="n"/>
       <c r="R5" s="11" t="n"/>
       <c r="S5" s="11" t="n"/>
       <c r="T5" s="11" t="n"/>
       <c r="U5" s="11" t="n"/>
       <c r="V5" s="11" t="n"/>
-      <c r="W5" s="11" t="n"/>
+      <c r="W5" s="11" t="n">
+        <v>41250.75</v>
+      </c>
       <c r="X5" s="11" t="n"/>
       <c r="Y5" s="11" t="n"/>
       <c r="Z5" s="11" t="n"/>
@@ -5874,27 +5657,21 @@
       <c r="G9" s="11" t="n"/>
       <c r="H9" s="11" t="n"/>
       <c r="I9" s="11" t="n"/>
-      <c r="J9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
+      <c r="J9" s="11" t="n"/>
       <c r="K9" s="11" t="n"/>
       <c r="L9" s="11" t="n"/>
       <c r="M9" s="11" t="n"/>
       <c r="N9" s="11" t="n"/>
       <c r="O9" s="11" t="n"/>
       <c r="P9" s="11" t="n"/>
-      <c r="Q9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
+      <c r="Q9" s="11" t="n"/>
       <c r="R9" s="11" t="n"/>
       <c r="S9" s="11" t="n"/>
       <c r="T9" s="11" t="n"/>
       <c r="U9" s="11" t="n"/>
       <c r="V9" s="11" t="n"/>
       <c r="W9" s="11" t="n"/>
-      <c r="X9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
+      <c r="X9" s="11" t="n"/>
       <c r="Y9" s="11" t="n"/>
       <c r="Z9" s="11" t="n"/>
       <c r="AA9" s="11" t="n"/>
@@ -5963,27 +5740,21 @@
       <c r="J11" s="11" t="n"/>
       <c r="K11" s="11" t="n"/>
       <c r="L11" s="11" t="n"/>
-      <c r="M11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
+      <c r="M11" s="11" t="n"/>
       <c r="N11" s="11" t="n"/>
       <c r="O11" s="11" t="n"/>
       <c r="P11" s="11" t="n"/>
       <c r="Q11" s="11" t="n"/>
       <c r="R11" s="11" t="n"/>
       <c r="S11" s="11" t="n"/>
-      <c r="T11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
+      <c r="T11" s="11" t="n"/>
       <c r="U11" s="11" t="n"/>
       <c r="V11" s="11" t="n"/>
       <c r="W11" s="11" t="n"/>
       <c r="X11" s="11" t="n"/>
       <c r="Y11" s="11" t="n"/>
       <c r="Z11" s="11" t="n"/>
-      <c r="AA11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
+      <c r="AA11" s="11" t="n"/>
       <c r="AB11" s="11" t="n"/>
       <c r="AC11" s="11" t="n"/>
       <c r="AD11" s="12">
@@ -6007,27 +5778,21 @@
       <c r="G12" s="11" t="n"/>
       <c r="H12" s="11" t="n"/>
       <c r="I12" s="11" t="n"/>
-      <c r="J12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
+      <c r="J12" s="11" t="n"/>
       <c r="K12" s="11" t="n"/>
       <c r="L12" s="11" t="n"/>
       <c r="M12" s="11" t="n"/>
       <c r="N12" s="11" t="n"/>
       <c r="O12" s="11" t="n"/>
       <c r="P12" s="11" t="n"/>
-      <c r="Q12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
+      <c r="Q12" s="11" t="n"/>
       <c r="R12" s="11" t="n"/>
       <c r="S12" s="11" t="n"/>
       <c r="T12" s="11" t="n"/>
       <c r="U12" s="11" t="n"/>
       <c r="V12" s="11" t="n"/>
       <c r="W12" s="11" t="n"/>
-      <c r="X12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
+      <c r="X12" s="11" t="n"/>
       <c r="Y12" s="11" t="n"/>
       <c r="Z12" s="11" t="n"/>
       <c r="AA12" s="11" t="n"/>
@@ -6055,27 +5820,21 @@
       <c r="H13" s="11" t="n"/>
       <c r="I13" s="11" t="n"/>
       <c r="J13" s="11" t="n"/>
-      <c r="K13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
+      <c r="K13" s="11" t="n"/>
       <c r="L13" s="11" t="n"/>
       <c r="M13" s="11" t="n"/>
       <c r="N13" s="11" t="n"/>
       <c r="O13" s="11" t="n"/>
       <c r="P13" s="11" t="n"/>
       <c r="Q13" s="11" t="n"/>
-      <c r="R13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
+      <c r="R13" s="11" t="n"/>
       <c r="S13" s="11" t="n"/>
       <c r="T13" s="11" t="n"/>
       <c r="U13" s="11" t="n"/>
       <c r="V13" s="11" t="n"/>
       <c r="W13" s="11" t="n"/>
       <c r="X13" s="11" t="n"/>
-      <c r="Y13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
+      <c r="Y13" s="11" t="n"/>
       <c r="Z13" s="11" t="n"/>
       <c r="AA13" s="11" t="n"/>
       <c r="AB13" s="11" t="n"/>
@@ -6103,27 +5862,21 @@
       <c r="I14" s="11" t="n"/>
       <c r="J14" s="11" t="n"/>
       <c r="K14" s="11" t="n"/>
-      <c r="L14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
+      <c r="L14" s="11" t="n"/>
       <c r="M14" s="11" t="n"/>
       <c r="N14" s="11" t="n"/>
       <c r="O14" s="11" t="n"/>
       <c r="P14" s="11" t="n"/>
       <c r="Q14" s="11" t="n"/>
       <c r="R14" s="11" t="n"/>
-      <c r="S14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
+      <c r="S14" s="11" t="n"/>
       <c r="T14" s="11" t="n"/>
       <c r="U14" s="11" t="n"/>
       <c r="V14" s="11" t="n"/>
       <c r="W14" s="11" t="n"/>
       <c r="X14" s="11" t="n"/>
       <c r="Y14" s="11" t="n"/>
-      <c r="Z14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
+      <c r="Z14" s="11" t="n"/>
       <c r="AA14" s="11" t="n"/>
       <c r="AB14" s="11" t="n"/>
       <c r="AC14" s="11" t="n"/>
@@ -6150,27 +5903,21 @@
       <c r="I15" s="11" t="n"/>
       <c r="J15" s="11" t="n"/>
       <c r="K15" s="11" t="n"/>
-      <c r="L15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
+      <c r="L15" s="11" t="n"/>
       <c r="M15" s="11" t="n"/>
       <c r="N15" s="11" t="n"/>
       <c r="O15" s="11" t="n"/>
       <c r="P15" s="11" t="n"/>
       <c r="Q15" s="11" t="n"/>
       <c r="R15" s="11" t="n"/>
-      <c r="S15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
+      <c r="S15" s="11" t="n"/>
       <c r="T15" s="11" t="n"/>
       <c r="U15" s="11" t="n"/>
       <c r="V15" s="11" t="n"/>
       <c r="W15" s="11" t="n"/>
       <c r="X15" s="11" t="n"/>
       <c r="Y15" s="11" t="n"/>
-      <c r="Z15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
+      <c r="Z15" s="11" t="n"/>
       <c r="AA15" s="11" t="n"/>
       <c r="AB15" s="11" t="n"/>
       <c r="AC15" s="11" t="n"/>
@@ -6296,16 +6043,16 @@
       <c r="M17" s="11" t="n"/>
       <c r="N17" s="11" t="n"/>
       <c r="O17" s="11" t="n"/>
-      <c r="P17" s="11" t="n"/>
+      <c r="P17" s="11" t="n">
+        <v>132834.8</v>
+      </c>
       <c r="Q17" s="11" t="n"/>
       <c r="R17" s="11" t="n"/>
       <c r="S17" s="11" t="n"/>
       <c r="T17" s="11" t="n"/>
       <c r="U17" s="11" t="n"/>
       <c r="V17" s="11" t="n"/>
-      <c r="W17" s="11" t="n">
-        <v>132834.8</v>
-      </c>
+      <c r="W17" s="11" t="n"/>
       <c r="X17" s="11" t="n"/>
       <c r="Y17" s="11" t="n"/>
       <c r="Z17" s="11" t="n"/>
@@ -6338,27 +6085,21 @@
       <c r="L18" s="11" t="n"/>
       <c r="M18" s="11" t="n"/>
       <c r="N18" s="11" t="n"/>
-      <c r="O18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
+      <c r="O18" s="11" t="n"/>
       <c r="P18" s="11" t="n"/>
       <c r="Q18" s="11" t="n"/>
       <c r="R18" s="11" t="n"/>
       <c r="S18" s="11" t="n"/>
       <c r="T18" s="11" t="n"/>
       <c r="U18" s="11" t="n"/>
-      <c r="V18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
+      <c r="V18" s="11" t="n"/>
       <c r="W18" s="11" t="n"/>
       <c r="X18" s="11" t="n"/>
       <c r="Y18" s="11" t="n"/>
       <c r="Z18" s="11" t="n"/>
       <c r="AA18" s="11" t="n"/>
       <c r="AB18" s="11" t="n"/>
-      <c r="AC18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
+      <c r="AC18" s="11" t="n"/>
       <c r="AD18" s="12">
         <f>SUM(B18:AC18)</f>
         <v/>
@@ -6380,27 +6121,21 @@
       <c r="G19" s="11" t="n"/>
       <c r="H19" s="11" t="n"/>
       <c r="I19" s="11" t="n"/>
-      <c r="J19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
+      <c r="J19" s="11" t="n"/>
       <c r="K19" s="11" t="n"/>
       <c r="L19" s="11" t="n"/>
       <c r="M19" s="11" t="n"/>
       <c r="N19" s="11" t="n"/>
       <c r="O19" s="11" t="n"/>
       <c r="P19" s="11" t="n"/>
-      <c r="Q19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
+      <c r="Q19" s="11" t="n"/>
       <c r="R19" s="11" t="n"/>
       <c r="S19" s="11" t="n"/>
       <c r="T19" s="11" t="n"/>
       <c r="U19" s="11" t="n"/>
       <c r="V19" s="11" t="n"/>
       <c r="W19" s="11" t="n"/>
-      <c r="X19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
+      <c r="X19" s="11" t="n"/>
       <c r="Y19" s="11" t="n"/>
       <c r="Z19" s="11" t="n"/>
       <c r="AA19" s="11" t="n"/>
@@ -6476,27 +6211,21 @@
       <c r="I21" s="11" t="n"/>
       <c r="J21" s="11" t="n"/>
       <c r="K21" s="11" t="n"/>
-      <c r="L21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
+      <c r="L21" s="11" t="n"/>
       <c r="M21" s="11" t="n"/>
       <c r="N21" s="11" t="n"/>
       <c r="O21" s="11" t="n"/>
       <c r="P21" s="11" t="n"/>
       <c r="Q21" s="11" t="n"/>
       <c r="R21" s="11" t="n"/>
-      <c r="S21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
+      <c r="S21" s="11" t="n"/>
       <c r="T21" s="11" t="n"/>
       <c r="U21" s="11" t="n"/>
       <c r="V21" s="11" t="n"/>
       <c r="W21" s="11" t="n"/>
       <c r="X21" s="11" t="n"/>
       <c r="Y21" s="11" t="n"/>
-      <c r="Z21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
+      <c r="Z21" s="11" t="n"/>
       <c r="AA21" s="11" t="n"/>
       <c r="AB21" s="11" t="n"/>
       <c r="AC21" s="11" t="n"/>
@@ -6523,27 +6252,21 @@
       <c r="I22" s="11" t="n"/>
       <c r="J22" s="11" t="n"/>
       <c r="K22" s="11" t="n"/>
-      <c r="L22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
+      <c r="L22" s="11" t="n"/>
       <c r="M22" s="11" t="n"/>
       <c r="N22" s="11" t="n"/>
       <c r="O22" s="11" t="n"/>
       <c r="P22" s="11" t="n"/>
       <c r="Q22" s="11" t="n"/>
       <c r="R22" s="11" t="n"/>
-      <c r="S22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
+      <c r="S22" s="11" t="n"/>
       <c r="T22" s="11" t="n"/>
       <c r="U22" s="11" t="n"/>
       <c r="V22" s="11" t="n"/>
       <c r="W22" s="11" t="n"/>
       <c r="X22" s="11" t="n"/>
       <c r="Y22" s="11" t="n"/>
-      <c r="Z22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
+      <c r="Z22" s="11" t="n"/>
       <c r="AA22" s="11" t="n"/>
       <c r="AB22" s="11" t="n"/>
       <c r="AC22" s="11" t="n"/>
@@ -7230,27 +6953,21 @@
       <c r="I3" s="11" t="n"/>
       <c r="J3" s="11" t="n"/>
       <c r="K3" s="11" t="n"/>
-      <c r="L3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
+      <c r="L3" s="11" t="n"/>
       <c r="M3" s="11" t="n"/>
       <c r="N3" s="11" t="n"/>
       <c r="O3" s="11" t="n"/>
       <c r="P3" s="11" t="n"/>
       <c r="Q3" s="11" t="n"/>
       <c r="R3" s="11" t="n"/>
-      <c r="S3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
+      <c r="S3" s="11" t="n"/>
       <c r="T3" s="11" t="n"/>
       <c r="U3" s="11" t="n"/>
       <c r="V3" s="11" t="n"/>
       <c r="W3" s="11" t="n"/>
       <c r="X3" s="11" t="n"/>
       <c r="Y3" s="11" t="n"/>
-      <c r="Z3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
+      <c r="Z3" s="11" t="n"/>
       <c r="AA3" s="11" t="n"/>
       <c r="AB3" s="11" t="n"/>
       <c r="AC3" s="11" t="n"/>
@@ -7310,32 +7027,32 @@
           <t>Sandwell MBC - Respite</t>
         </is>
       </c>
-      <c r="B5" s="11" t="n">
-        <v>41250.75</v>
-      </c>
+      <c r="B5" s="11" t="n"/>
       <c r="C5" s="11" t="n"/>
       <c r="D5" s="11" t="n"/>
       <c r="E5" s="11" t="n"/>
       <c r="F5" s="11" t="n"/>
       <c r="G5" s="11" t="n"/>
       <c r="H5" s="11" t="n"/>
-      <c r="I5" s="11" t="n"/>
+      <c r="I5" s="11" t="n">
+        <v>41250.75</v>
+      </c>
       <c r="J5" s="11" t="n"/>
       <c r="K5" s="11" t="n"/>
       <c r="L5" s="11" t="n"/>
       <c r="M5" s="11" t="n"/>
       <c r="N5" s="11" t="n"/>
       <c r="O5" s="11" t="n"/>
-      <c r="P5" s="11" t="n">
-        <v>41250.75</v>
-      </c>
+      <c r="P5" s="11" t="n"/>
       <c r="Q5" s="11" t="n"/>
       <c r="R5" s="11" t="n"/>
       <c r="S5" s="11" t="n"/>
       <c r="T5" s="11" t="n"/>
       <c r="U5" s="11" t="n"/>
       <c r="V5" s="11" t="n"/>
-      <c r="W5" s="11" t="n"/>
+      <c r="W5" s="11" t="n">
+        <v>41250.75</v>
+      </c>
       <c r="X5" s="11" t="n"/>
       <c r="Y5" s="11" t="n"/>
       <c r="Z5" s="11" t="n"/>
@@ -7504,27 +7221,21 @@
       <c r="G9" s="11" t="n"/>
       <c r="H9" s="11" t="n"/>
       <c r="I9" s="11" t="n"/>
-      <c r="J9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
+      <c r="J9" s="11" t="n"/>
       <c r="K9" s="11" t="n"/>
       <c r="L9" s="11" t="n"/>
       <c r="M9" s="11" t="n"/>
       <c r="N9" s="11" t="n"/>
       <c r="O9" s="11" t="n"/>
       <c r="P9" s="11" t="n"/>
-      <c r="Q9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
+      <c r="Q9" s="11" t="n"/>
       <c r="R9" s="11" t="n"/>
       <c r="S9" s="11" t="n"/>
       <c r="T9" s="11" t="n"/>
       <c r="U9" s="11" t="n"/>
       <c r="V9" s="11" t="n"/>
       <c r="W9" s="11" t="n"/>
-      <c r="X9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
+      <c r="X9" s="11" t="n"/>
       <c r="Y9" s="11" t="n"/>
       <c r="Z9" s="11" t="n"/>
       <c r="AA9" s="11" t="n"/>
@@ -7601,27 +7312,21 @@
       <c r="J11" s="11" t="n"/>
       <c r="K11" s="11" t="n"/>
       <c r="L11" s="11" t="n"/>
-      <c r="M11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
+      <c r="M11" s="11" t="n"/>
       <c r="N11" s="11" t="n"/>
       <c r="O11" s="11" t="n"/>
       <c r="P11" s="11" t="n"/>
       <c r="Q11" s="11" t="n"/>
       <c r="R11" s="11" t="n"/>
       <c r="S11" s="11" t="n"/>
-      <c r="T11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
+      <c r="T11" s="11" t="n"/>
       <c r="U11" s="11" t="n"/>
       <c r="V11" s="11" t="n"/>
       <c r="W11" s="11" t="n"/>
       <c r="X11" s="11" t="n"/>
       <c r="Y11" s="11" t="n"/>
       <c r="Z11" s="11" t="n"/>
-      <c r="AA11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
+      <c r="AA11" s="11" t="n"/>
       <c r="AB11" s="11" t="n"/>
       <c r="AC11" s="11" t="n"/>
       <c r="AD11" s="11" t="n"/>
@@ -7648,27 +7353,21 @@
       <c r="G12" s="11" t="n"/>
       <c r="H12" s="11" t="n"/>
       <c r="I12" s="11" t="n"/>
-      <c r="J12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
+      <c r="J12" s="11" t="n"/>
       <c r="K12" s="11" t="n"/>
       <c r="L12" s="11" t="n"/>
       <c r="M12" s="11" t="n"/>
       <c r="N12" s="11" t="n"/>
       <c r="O12" s="11" t="n"/>
       <c r="P12" s="11" t="n"/>
-      <c r="Q12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
+      <c r="Q12" s="11" t="n"/>
       <c r="R12" s="11" t="n"/>
       <c r="S12" s="11" t="n"/>
       <c r="T12" s="11" t="n"/>
       <c r="U12" s="11" t="n"/>
       <c r="V12" s="11" t="n"/>
       <c r="W12" s="11" t="n"/>
-      <c r="X12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
+      <c r="X12" s="11" t="n"/>
       <c r="Y12" s="11" t="n"/>
       <c r="Z12" s="11" t="n"/>
       <c r="AA12" s="11" t="n"/>
@@ -7701,27 +7400,21 @@
       <c r="H13" s="11" t="n"/>
       <c r="I13" s="11" t="n"/>
       <c r="J13" s="11" t="n"/>
-      <c r="K13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
+      <c r="K13" s="11" t="n"/>
       <c r="L13" s="11" t="n"/>
       <c r="M13" s="11" t="n"/>
       <c r="N13" s="11" t="n"/>
       <c r="O13" s="11" t="n"/>
       <c r="P13" s="11" t="n"/>
       <c r="Q13" s="11" t="n"/>
-      <c r="R13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
+      <c r="R13" s="11" t="n"/>
       <c r="S13" s="11" t="n"/>
       <c r="T13" s="11" t="n"/>
       <c r="U13" s="11" t="n"/>
       <c r="V13" s="11" t="n"/>
       <c r="W13" s="11" t="n"/>
       <c r="X13" s="11" t="n"/>
-      <c r="Y13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
+      <c r="Y13" s="11" t="n"/>
       <c r="Z13" s="11" t="n"/>
       <c r="AA13" s="11" t="n"/>
       <c r="AB13" s="11" t="n"/>
@@ -7754,27 +7447,21 @@
       <c r="I14" s="11" t="n"/>
       <c r="J14" s="11" t="n"/>
       <c r="K14" s="11" t="n"/>
-      <c r="L14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
+      <c r="L14" s="11" t="n"/>
       <c r="M14" s="11" t="n"/>
       <c r="N14" s="11" t="n"/>
       <c r="O14" s="11" t="n"/>
       <c r="P14" s="11" t="n"/>
       <c r="Q14" s="11" t="n"/>
       <c r="R14" s="11" t="n"/>
-      <c r="S14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
+      <c r="S14" s="11" t="n"/>
       <c r="T14" s="11" t="n"/>
       <c r="U14" s="11" t="n"/>
       <c r="V14" s="11" t="n"/>
       <c r="W14" s="11" t="n"/>
       <c r="X14" s="11" t="n"/>
       <c r="Y14" s="11" t="n"/>
-      <c r="Z14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
+      <c r="Z14" s="11" t="n"/>
       <c r="AA14" s="11" t="n"/>
       <c r="AB14" s="11" t="n"/>
       <c r="AC14" s="11" t="n"/>
@@ -7804,27 +7491,21 @@
       <c r="I15" s="11" t="n"/>
       <c r="J15" s="11" t="n"/>
       <c r="K15" s="11" t="n"/>
-      <c r="L15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
+      <c r="L15" s="11" t="n"/>
       <c r="M15" s="11" t="n"/>
       <c r="N15" s="11" t="n"/>
       <c r="O15" s="11" t="n"/>
       <c r="P15" s="11" t="n"/>
       <c r="Q15" s="11" t="n"/>
       <c r="R15" s="11" t="n"/>
-      <c r="S15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
+      <c r="S15" s="11" t="n"/>
       <c r="T15" s="11" t="n"/>
       <c r="U15" s="11" t="n"/>
       <c r="V15" s="11" t="n"/>
       <c r="W15" s="11" t="n"/>
       <c r="X15" s="11" t="n"/>
       <c r="Y15" s="11" t="n"/>
-      <c r="Z15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
+      <c r="Z15" s="11" t="n"/>
       <c r="AA15" s="11" t="n"/>
       <c r="AB15" s="11" t="n"/>
       <c r="AC15" s="11" t="n"/>
@@ -7962,23 +7643,25 @@
       <c r="M17" s="11" t="n"/>
       <c r="N17" s="11" t="n"/>
       <c r="O17" s="11" t="n"/>
-      <c r="P17" s="11" t="n"/>
+      <c r="P17" s="11" t="n">
+        <v>132834.8</v>
+      </c>
       <c r="Q17" s="11" t="n"/>
       <c r="R17" s="11" t="n"/>
       <c r="S17" s="11" t="n"/>
       <c r="T17" s="11" t="n"/>
       <c r="U17" s="11" t="n"/>
       <c r="V17" s="11" t="n"/>
-      <c r="W17" s="11" t="n">
-        <v>132834.8</v>
-      </c>
+      <c r="W17" s="11" t="n"/>
       <c r="X17" s="11" t="n"/>
       <c r="Y17" s="11" t="n"/>
       <c r="Z17" s="11" t="n"/>
       <c r="AA17" s="11" t="n"/>
       <c r="AB17" s="11" t="n"/>
       <c r="AC17" s="11" t="n"/>
-      <c r="AD17" s="11" t="n"/>
+      <c r="AD17" s="11" t="n">
+        <v>132834.8</v>
+      </c>
       <c r="AE17" s="11" t="n"/>
       <c r="AF17" s="11" t="n"/>
       <c r="AG17" s="12">
@@ -8007,27 +7690,21 @@
       <c r="L18" s="11" t="n"/>
       <c r="M18" s="11" t="n"/>
       <c r="N18" s="11" t="n"/>
-      <c r="O18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
+      <c r="O18" s="11" t="n"/>
       <c r="P18" s="11" t="n"/>
       <c r="Q18" s="11" t="n"/>
       <c r="R18" s="11" t="n"/>
       <c r="S18" s="11" t="n"/>
       <c r="T18" s="11" t="n"/>
       <c r="U18" s="11" t="n"/>
-      <c r="V18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
+      <c r="V18" s="11" t="n"/>
       <c r="W18" s="11" t="n"/>
       <c r="X18" s="11" t="n"/>
       <c r="Y18" s="11" t="n"/>
       <c r="Z18" s="11" t="n"/>
       <c r="AA18" s="11" t="n"/>
       <c r="AB18" s="11" t="n"/>
-      <c r="AC18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
+      <c r="AC18" s="11" t="n"/>
       <c r="AD18" s="11" t="n"/>
       <c r="AE18" s="11" t="n"/>
       <c r="AF18" s="11" t="n"/>
@@ -8052,27 +7729,21 @@
       <c r="G19" s="11" t="n"/>
       <c r="H19" s="11" t="n"/>
       <c r="I19" s="11" t="n"/>
-      <c r="J19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
+      <c r="J19" s="11" t="n"/>
       <c r="K19" s="11" t="n"/>
       <c r="L19" s="11" t="n"/>
       <c r="M19" s="11" t="n"/>
       <c r="N19" s="11" t="n"/>
       <c r="O19" s="11" t="n"/>
       <c r="P19" s="11" t="n"/>
-      <c r="Q19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
+      <c r="Q19" s="11" t="n"/>
       <c r="R19" s="11" t="n"/>
       <c r="S19" s="11" t="n"/>
       <c r="T19" s="11" t="n"/>
       <c r="U19" s="11" t="n"/>
       <c r="V19" s="11" t="n"/>
       <c r="W19" s="11" t="n"/>
-      <c r="X19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
+      <c r="X19" s="11" t="n"/>
       <c r="Y19" s="11" t="n"/>
       <c r="Z19" s="11" t="n"/>
       <c r="AA19" s="11" t="n"/>
@@ -8156,27 +7827,21 @@
       <c r="I21" s="11" t="n"/>
       <c r="J21" s="11" t="n"/>
       <c r="K21" s="11" t="n"/>
-      <c r="L21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
+      <c r="L21" s="11" t="n"/>
       <c r="M21" s="11" t="n"/>
       <c r="N21" s="11" t="n"/>
       <c r="O21" s="11" t="n"/>
       <c r="P21" s="11" t="n"/>
       <c r="Q21" s="11" t="n"/>
       <c r="R21" s="11" t="n"/>
-      <c r="S21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
+      <c r="S21" s="11" t="n"/>
       <c r="T21" s="11" t="n"/>
       <c r="U21" s="11" t="n"/>
       <c r="V21" s="11" t="n"/>
       <c r="W21" s="11" t="n"/>
       <c r="X21" s="11" t="n"/>
       <c r="Y21" s="11" t="n"/>
-      <c r="Z21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
+      <c r="Z21" s="11" t="n"/>
       <c r="AA21" s="11" t="n"/>
       <c r="AB21" s="11" t="n"/>
       <c r="AC21" s="11" t="n"/>
@@ -8206,27 +7871,21 @@
       <c r="I22" s="11" t="n"/>
       <c r="J22" s="11" t="n"/>
       <c r="K22" s="11" t="n"/>
-      <c r="L22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
+      <c r="L22" s="11" t="n"/>
       <c r="M22" s="11" t="n"/>
       <c r="N22" s="11" t="n"/>
       <c r="O22" s="11" t="n"/>
       <c r="P22" s="11" t="n"/>
       <c r="Q22" s="11" t="n"/>
       <c r="R22" s="11" t="n"/>
-      <c r="S22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
+      <c r="S22" s="11" t="n"/>
       <c r="T22" s="11" t="n"/>
       <c r="U22" s="11" t="n"/>
       <c r="V22" s="11" t="n"/>
       <c r="W22" s="11" t="n"/>
       <c r="X22" s="11" t="n"/>
       <c r="Y22" s="11" t="n"/>
-      <c r="Z22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
+      <c r="Z22" s="11" t="n"/>
       <c r="AA22" s="11" t="n"/>
       <c r="AB22" s="11" t="n"/>
       <c r="AC22" s="11" t="n"/>
@@ -12398,15 +12057,9 @@
           <t>Birmingham City Council - Supported Living</t>
         </is>
       </c>
-      <c r="E3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
-      <c r="L3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
-      <c r="S3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
+      <c r="E3" s="11" t="n"/>
+      <c r="L3" s="11" t="n"/>
+      <c r="S3" s="11" t="n"/>
       <c r="Z3" s="11" t="n">
         <v>59419.08</v>
       </c>
@@ -12438,6 +12091,9 @@
       <c r="P5" s="11" t="n">
         <v>41250.75</v>
       </c>
+      <c r="AD5" s="11" t="n">
+        <v>41250.75</v>
+      </c>
       <c r="AF5" s="12">
         <f>SUM(B5:AE5)</f>
         <v/>
@@ -12449,10 +12105,12 @@
           <t>Sandwell MBC - Daycare</t>
         </is>
       </c>
-      <c r="F6" s="11" t="n">
+      <c r="F6" s="11" t="n"/>
+      <c r="M6" s="11" t="n">
         <v>6585.35</v>
       </c>
-      <c r="T6" s="11" t="n">
+      <c r="T6" s="11" t="n"/>
+      <c r="AA6" s="11" t="n">
         <v>6585.35</v>
       </c>
       <c r="AF6" s="12">
@@ -12500,21 +12158,13 @@
           <t>Walsall - Respite</t>
         </is>
       </c>
-      <c r="C9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
-      <c r="J9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
-      <c r="Q9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
+      <c r="C9" s="11" t="n"/>
+      <c r="J9" s="11" t="n"/>
+      <c r="Q9" s="11" t="n"/>
       <c r="X9" s="11" t="n">
         <v>11460.8</v>
       </c>
-      <c r="AE9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
+      <c r="AE9" s="11" t="n"/>
       <c r="AF9" s="12">
         <f>SUM(B9:AE9)</f>
         <v/>
@@ -12537,15 +12187,9 @@
           <t>Ideal for All Ltd - Direct Payments</t>
         </is>
       </c>
-      <c r="F11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
-      <c r="M11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
-      <c r="T11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
+      <c r="F11" s="11" t="n"/>
+      <c r="M11" s="11" t="n"/>
+      <c r="T11" s="11" t="n"/>
       <c r="AA11" s="11" t="n">
         <v>4131.62</v>
       </c>
@@ -12560,21 +12204,13 @@
           <t>Kirklees - Supported Living</t>
         </is>
       </c>
-      <c r="C12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
-      <c r="J12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
-      <c r="Q12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
+      <c r="C12" s="11" t="n"/>
+      <c r="J12" s="11" t="n"/>
+      <c r="Q12" s="11" t="n"/>
       <c r="X12" s="11" t="n">
         <v>5458.48</v>
       </c>
-      <c r="AE12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
+      <c r="AE12" s="11" t="n"/>
       <c r="AF12" s="12">
         <f>SUM(B12:AE12)</f>
         <v/>
@@ -12586,15 +12222,9 @@
           <t>LB Hillingdon - Supported Living</t>
         </is>
       </c>
-      <c r="D13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
-      <c r="K13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
-      <c r="R13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
+      <c r="D13" s="11" t="n"/>
+      <c r="K13" s="11" t="n"/>
+      <c r="R13" s="11" t="n"/>
       <c r="Y13" s="11" t="n">
         <v>5203.8</v>
       </c>
@@ -12609,15 +12239,9 @@
           <t>NHS Birmingham &amp; Solihull ICB</t>
         </is>
       </c>
-      <c r="E14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
-      <c r="L14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
-      <c r="S14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
+      <c r="E14" s="11" t="n"/>
+      <c r="L14" s="11" t="n"/>
+      <c r="S14" s="11" t="n"/>
       <c r="Z14" s="11" t="n">
         <v>7814.17</v>
       </c>
@@ -12632,15 +12256,9 @@
           <t>NHS Black Country ICB</t>
         </is>
       </c>
-      <c r="E15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
-      <c r="L15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
-      <c r="S15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
+      <c r="E15" s="11" t="n"/>
+      <c r="L15" s="11" t="n"/>
+      <c r="S15" s="11" t="n"/>
       <c r="Z15" s="11" t="n">
         <v>5499.45</v>
       </c>
@@ -12756,7 +12374,8 @@
           <t>Sandwell MBC - Supported Living</t>
         </is>
       </c>
-      <c r="B17" s="11" t="n">
+      <c r="B17" s="11" t="n"/>
+      <c r="I17" s="11" t="n">
         <v>132834.8</v>
       </c>
       <c r="W17" s="11" t="n">
@@ -12773,15 +12392,9 @@
           <t>Solihull MBC - Supported Living</t>
         </is>
       </c>
-      <c r="H18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
-      <c r="O18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
-      <c r="V18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
+      <c r="H18" s="11" t="n"/>
+      <c r="O18" s="11" t="n"/>
+      <c r="V18" s="11" t="n"/>
       <c r="AC18" s="11" t="n">
         <v>33031.6</v>
       </c>
@@ -12796,21 +12409,13 @@
           <t>Walsall - Supported Living</t>
         </is>
       </c>
-      <c r="C19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
-      <c r="J19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
-      <c r="Q19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
+      <c r="C19" s="11" t="n"/>
+      <c r="J19" s="11" t="n"/>
+      <c r="Q19" s="11" t="n"/>
       <c r="X19" s="11" t="n">
         <v>319655.76</v>
       </c>
-      <c r="AE19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
+      <c r="AE19" s="11" t="n"/>
       <c r="AF19" s="12">
         <f>SUM(B19:AE19)</f>
         <v/>
@@ -12845,15 +12450,9 @@
           <t>People Plus - Direct Payments</t>
         </is>
       </c>
-      <c r="E21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
-      <c r="L21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
-      <c r="S21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
+      <c r="E21" s="11" t="n"/>
+      <c r="L21" s="11" t="n"/>
+      <c r="S21" s="11" t="n"/>
       <c r="Z21" s="11" t="n">
         <v>21527.2</v>
       </c>
@@ -12868,15 +12467,9 @@
           <t>Middlesbrough - Supported Living</t>
         </is>
       </c>
-      <c r="E22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
-      <c r="L22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
-      <c r="S22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
+      <c r="E22" s="11" t="n"/>
+      <c r="L22" s="11" t="n"/>
+      <c r="S22" s="11" t="n"/>
       <c r="Z22" s="11" t="n">
         <v>6115.4</v>
       </c>
@@ -13544,21 +13137,13 @@
           <t>Birmingham City Council - Supported Living</t>
         </is>
       </c>
-      <c r="C3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
-      <c r="J3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
-      <c r="Q3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
+      <c r="C3" s="11" t="n"/>
+      <c r="J3" s="11" t="n"/>
+      <c r="Q3" s="11" t="n"/>
       <c r="X3" s="11" t="n">
         <v>59419.08</v>
       </c>
-      <c r="AE3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
+      <c r="AE3" s="11" t="n"/>
       <c r="AG3" s="12">
         <f>SUM(B3:AF3)</f>
         <v/>
@@ -13581,10 +13166,12 @@
           <t>Sandwell MBC - Respite</t>
         </is>
       </c>
-      <c r="G5" s="11" t="n">
+      <c r="G5" s="11" t="n"/>
+      <c r="N5" s="11" t="n">
         <v>41250.75</v>
       </c>
-      <c r="U5" s="11" t="n">
+      <c r="U5" s="11" t="n"/>
+      <c r="AB5" s="11" t="n">
         <v>41250.75</v>
       </c>
       <c r="AG5" s="12">
@@ -13598,10 +13185,12 @@
           <t>Sandwell MBC - Daycare</t>
         </is>
       </c>
-      <c r="D6" s="11" t="n">
+      <c r="D6" s="11" t="n"/>
+      <c r="K6" s="11" t="n">
         <v>6585.35</v>
       </c>
-      <c r="R6" s="11" t="n">
+      <c r="R6" s="11" t="n"/>
+      <c r="Y6" s="11" t="n">
         <v>6585.35</v>
       </c>
       <c r="AG6" s="12">
@@ -13652,18 +13241,12 @@
           <t>Walsall - Respite</t>
         </is>
       </c>
-      <c r="H9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
-      <c r="O9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
+      <c r="H9" s="11" t="n"/>
+      <c r="O9" s="11" t="n"/>
       <c r="V9" s="11" t="n">
         <v>11460.8</v>
       </c>
-      <c r="AC9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
+      <c r="AC9" s="11" t="n"/>
       <c r="AG9" s="12">
         <f>SUM(B9:AF9)</f>
         <v/>
@@ -13686,21 +13269,13 @@
           <t>Ideal for All Ltd - Direct Payments</t>
         </is>
       </c>
-      <c r="D11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
-      <c r="K11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
-      <c r="R11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
+      <c r="D11" s="11" t="n"/>
+      <c r="K11" s="11" t="n"/>
+      <c r="R11" s="11" t="n"/>
       <c r="Y11" s="11" t="n">
         <v>4131.62</v>
       </c>
-      <c r="AF11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
+      <c r="AF11" s="11" t="n"/>
       <c r="AG11" s="12">
         <f>SUM(B11:AF11)</f>
         <v/>
@@ -13712,18 +13287,12 @@
           <t>Kirklees - Supported Living</t>
         </is>
       </c>
-      <c r="H12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
-      <c r="O12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
+      <c r="H12" s="11" t="n"/>
+      <c r="O12" s="11" t="n"/>
       <c r="V12" s="11" t="n">
         <v>5458.48</v>
       </c>
-      <c r="AC12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
+      <c r="AC12" s="11" t="n"/>
       <c r="AG12" s="12">
         <f>SUM(B12:AF12)</f>
         <v/>
@@ -13735,21 +13304,13 @@
           <t>LB Hillingdon - Supported Living</t>
         </is>
       </c>
-      <c r="B13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
-      <c r="I13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
-      <c r="P13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
+      <c r="B13" s="11" t="n"/>
+      <c r="I13" s="11" t="n"/>
+      <c r="P13" s="11" t="n"/>
       <c r="W13" s="11" t="n">
         <v>5203.8</v>
       </c>
-      <c r="AD13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
+      <c r="AD13" s="11" t="n"/>
       <c r="AG13" s="12">
         <f>SUM(B13:AF13)</f>
         <v/>
@@ -13761,21 +13322,13 @@
           <t>NHS Birmingham &amp; Solihull ICB</t>
         </is>
       </c>
-      <c r="C14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
-      <c r="J14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
-      <c r="Q14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
+      <c r="C14" s="11" t="n"/>
+      <c r="J14" s="11" t="n"/>
+      <c r="Q14" s="11" t="n"/>
       <c r="X14" s="11" t="n">
         <v>7814.17</v>
       </c>
-      <c r="AE14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
+      <c r="AE14" s="11" t="n"/>
       <c r="AG14" s="12">
         <f>SUM(B14:AF14)</f>
         <v/>
@@ -13787,21 +13340,13 @@
           <t>NHS Black Country ICB</t>
         </is>
       </c>
-      <c r="C15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
-      <c r="J15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
-      <c r="Q15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
+      <c r="C15" s="11" t="n"/>
+      <c r="J15" s="11" t="n"/>
+      <c r="Q15" s="11" t="n"/>
       <c r="X15" s="11" t="n">
         <v>5499.45</v>
       </c>
-      <c r="AE15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
+      <c r="AE15" s="11" t="n"/>
       <c r="AG15" s="12">
         <f>SUM(B15:AF15)</f>
         <v/>
@@ -13920,9 +13465,10 @@
       <c r="G17" s="11" t="n">
         <v>132834.8</v>
       </c>
-      <c r="AB17" s="11" t="n">
+      <c r="U17" s="11" t="n">
         <v>132834.8</v>
       </c>
+      <c r="AB17" s="11" t="n"/>
       <c r="AG17" s="12">
         <f>SUM(B17:AF17)</f>
         <v/>
@@ -13934,15 +13480,9 @@
           <t>Solihull MBC - Supported Living</t>
         </is>
       </c>
-      <c r="F18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
-      <c r="M18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
-      <c r="T18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
+      <c r="F18" s="11" t="n"/>
+      <c r="M18" s="11" t="n"/>
+      <c r="T18" s="11" t="n"/>
       <c r="AA18" s="11" t="n">
         <v>33031.6</v>
       </c>
@@ -13957,18 +13497,12 @@
           <t>Walsall - Supported Living</t>
         </is>
       </c>
-      <c r="H19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
-      <c r="O19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
+      <c r="H19" s="11" t="n"/>
+      <c r="O19" s="11" t="n"/>
       <c r="V19" s="11" t="n">
         <v>319655.76</v>
       </c>
-      <c r="AC19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
+      <c r="AC19" s="11" t="n"/>
       <c r="AG19" s="12">
         <f>SUM(B19:AF19)</f>
         <v/>
@@ -14006,21 +13540,13 @@
           <t>People Plus - Direct Payments</t>
         </is>
       </c>
-      <c r="C21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
-      <c r="J21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
-      <c r="Q21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
+      <c r="C21" s="11" t="n"/>
+      <c r="J21" s="11" t="n"/>
+      <c r="Q21" s="11" t="n"/>
       <c r="X21" s="11" t="n">
         <v>21527.2</v>
       </c>
-      <c r="AE21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
+      <c r="AE21" s="11" t="n"/>
       <c r="AG21" s="12">
         <f>SUM(B21:AF21)</f>
         <v/>
@@ -14032,21 +13558,13 @@
           <t>Middlesbrough - Supported Living</t>
         </is>
       </c>
-      <c r="C22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
-      <c r="J22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
-      <c r="Q22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
+      <c r="C22" s="11" t="n"/>
+      <c r="J22" s="11" t="n"/>
+      <c r="Q22" s="11" t="n"/>
       <c r="X22" s="11" t="n">
         <v>6115.4</v>
       </c>
-      <c r="AE22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
+      <c r="AE22" s="11" t="n"/>
       <c r="AG22" s="12">
         <f>SUM(B22:AF22)</f>
         <v/>
@@ -14721,18 +14239,12 @@
           <t>Birmingham City Council - Supported Living</t>
         </is>
       </c>
-      <c r="G3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
-      <c r="N3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
+      <c r="G3" s="11" t="n"/>
+      <c r="N3" s="11" t="n"/>
       <c r="U3" s="11" t="n">
         <v>59419.08</v>
       </c>
-      <c r="AB3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
+      <c r="AB3" s="11" t="n"/>
       <c r="AG3" s="12">
         <f>SUM(B3:AF3)</f>
         <v/>
@@ -14755,10 +14267,12 @@
           <t>Sandwell MBC - Respite</t>
         </is>
       </c>
-      <c r="D5" s="11" t="n">
+      <c r="D5" s="11" t="n"/>
+      <c r="K5" s="11" t="n">
         <v>41250.75</v>
       </c>
-      <c r="R5" s="11" t="n">
+      <c r="R5" s="11" t="n"/>
+      <c r="Y5" s="11" t="n">
         <v>41250.75</v>
       </c>
       <c r="AG5" s="12">
@@ -14823,18 +14337,12 @@
           <t>Walsall - Respite</t>
         </is>
       </c>
-      <c r="E9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
-      <c r="L9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
+      <c r="E9" s="11" t="n"/>
+      <c r="L9" s="11" t="n"/>
       <c r="S9" s="11" t="n">
         <v>11460.8</v>
       </c>
-      <c r="Z9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
+      <c r="Z9" s="11" t="n"/>
       <c r="AG9" s="12">
         <f>SUM(B9:AF9)</f>
         <v/>
@@ -14857,18 +14365,12 @@
           <t>Ideal for All Ltd - Direct Payments</t>
         </is>
       </c>
-      <c r="H11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
-      <c r="O11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
+      <c r="H11" s="11" t="n"/>
+      <c r="O11" s="11" t="n"/>
       <c r="V11" s="11" t="n">
         <v>4131.62</v>
       </c>
-      <c r="AC11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
+      <c r="AC11" s="11" t="n"/>
       <c r="AG11" s="12">
         <f>SUM(B11:AF11)</f>
         <v/>
@@ -14880,18 +14382,12 @@
           <t>Kirklees - Supported Living</t>
         </is>
       </c>
-      <c r="E12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
-      <c r="L12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
+      <c r="E12" s="11" t="n"/>
+      <c r="L12" s="11" t="n"/>
       <c r="S12" s="11" t="n">
         <v>5458.48</v>
       </c>
-      <c r="Z12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
+      <c r="Z12" s="11" t="n"/>
       <c r="AG12" s="12">
         <f>SUM(B12:AF12)</f>
         <v/>
@@ -14903,18 +14399,12 @@
           <t>LB Hillingdon - Supported Living</t>
         </is>
       </c>
-      <c r="F13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
-      <c r="M13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
+      <c r="F13" s="11" t="n"/>
+      <c r="M13" s="11" t="n"/>
       <c r="T13" s="11" t="n">
         <v>5203.8</v>
       </c>
-      <c r="AA13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
+      <c r="AA13" s="11" t="n"/>
       <c r="AG13" s="12">
         <f>SUM(B13:AF13)</f>
         <v/>
@@ -14926,18 +14416,12 @@
           <t>NHS Birmingham &amp; Solihull ICB</t>
         </is>
       </c>
-      <c r="G14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
-      <c r="N14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
+      <c r="G14" s="11" t="n"/>
+      <c r="N14" s="11" t="n"/>
       <c r="U14" s="11" t="n">
         <v>7814.17</v>
       </c>
-      <c r="AB14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
+      <c r="AB14" s="11" t="n"/>
       <c r="AG14" s="12">
         <f>SUM(B14:AF14)</f>
         <v/>
@@ -14949,18 +14433,12 @@
           <t>NHS Black Country ICB</t>
         </is>
       </c>
-      <c r="G15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
-      <c r="N15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
+      <c r="G15" s="11" t="n"/>
+      <c r="N15" s="11" t="n"/>
       <c r="U15" s="11" t="n">
         <v>5499.45</v>
       </c>
-      <c r="AB15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
+      <c r="AB15" s="11" t="n"/>
       <c r="AG15" s="12">
         <f>SUM(B15:AF15)</f>
         <v/>
@@ -15079,7 +14557,11 @@
       <c r="D17" s="11" t="n">
         <v>132834.8</v>
       </c>
-      <c r="Y17" s="11" t="n">
+      <c r="R17" s="11" t="n">
+        <v>132834.8</v>
+      </c>
+      <c r="Y17" s="11" t="n"/>
+      <c r="AF17" s="11" t="n">
         <v>132834.8</v>
       </c>
       <c r="AG17" s="12">
@@ -15093,21 +14575,13 @@
           <t>Solihull MBC - Supported Living</t>
         </is>
       </c>
-      <c r="C18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
-      <c r="J18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
-      <c r="Q18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
+      <c r="C18" s="11" t="n"/>
+      <c r="J18" s="11" t="n"/>
+      <c r="Q18" s="11" t="n"/>
       <c r="X18" s="11" t="n">
         <v>33031.6</v>
       </c>
-      <c r="AE18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
+      <c r="AE18" s="11" t="n"/>
       <c r="AG18" s="12">
         <f>SUM(B18:AF18)</f>
         <v/>
@@ -15119,18 +14593,12 @@
           <t>Walsall - Supported Living</t>
         </is>
       </c>
-      <c r="E19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
-      <c r="L19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
+      <c r="E19" s="11" t="n"/>
+      <c r="L19" s="11" t="n"/>
       <c r="S19" s="11" t="n">
         <v>319655.76</v>
       </c>
-      <c r="Z19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
+      <c r="Z19" s="11" t="n"/>
       <c r="AG19" s="12">
         <f>SUM(B19:AF19)</f>
         <v/>
@@ -15165,18 +14633,12 @@
           <t>People Plus - Direct Payments</t>
         </is>
       </c>
-      <c r="G21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
-      <c r="N21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
+      <c r="G21" s="11" t="n"/>
+      <c r="N21" s="11" t="n"/>
       <c r="U21" s="11" t="n">
         <v>21527.2</v>
       </c>
-      <c r="AB21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
+      <c r="AB21" s="11" t="n"/>
       <c r="AG21" s="12">
         <f>SUM(B21:AF21)</f>
         <v/>
@@ -15188,18 +14650,12 @@
           <t>Middlesbrough - Supported Living</t>
         </is>
       </c>
-      <c r="G22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
-      <c r="N22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
+      <c r="G22" s="11" t="n"/>
+      <c r="N22" s="11" t="n"/>
       <c r="U22" s="11" t="n">
         <v>6115.4</v>
       </c>
-      <c r="AB22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
+      <c r="AB22" s="11" t="n"/>
       <c r="AG22" s="12">
         <f>SUM(B22:AF22)</f>
         <v/>
@@ -15865,18 +15321,12 @@
           <t>Birmingham City Council - Supported Living</t>
         </is>
       </c>
-      <c r="D3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
-      <c r="K3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
+      <c r="D3" s="11" t="n"/>
+      <c r="K3" s="11" t="n"/>
       <c r="R3" s="11" t="n">
         <v>59419.08</v>
       </c>
-      <c r="Y3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
+      <c r="Y3" s="11" t="n"/>
       <c r="AF3" s="12">
         <f>SUM(B3:AE3)</f>
         <v/>
@@ -15967,21 +15417,13 @@
           <t>Walsall - Respite</t>
         </is>
       </c>
-      <c r="B9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
-      <c r="I9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
+      <c r="B9" s="11" t="n"/>
+      <c r="I9" s="11" t="n"/>
       <c r="P9" s="11" t="n">
         <v>11460.8</v>
       </c>
-      <c r="W9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
-      <c r="AD9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
+      <c r="W9" s="11" t="n"/>
+      <c r="AD9" s="11" t="n"/>
       <c r="AF9" s="12">
         <f>SUM(B9:AE9)</f>
         <v/>
@@ -16004,18 +15446,12 @@
           <t>Ideal for All Ltd - Direct Payments</t>
         </is>
       </c>
-      <c r="E11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
-      <c r="L11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
+      <c r="E11" s="11" t="n"/>
+      <c r="L11" s="11" t="n"/>
       <c r="S11" s="11" t="n">
         <v>4131.62</v>
       </c>
-      <c r="Z11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
+      <c r="Z11" s="11" t="n"/>
       <c r="AF11" s="12">
         <f>SUM(B11:AE11)</f>
         <v/>
@@ -16027,21 +15463,13 @@
           <t>Kirklees - Supported Living</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
-      <c r="I12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
+      <c r="B12" s="11" t="n"/>
+      <c r="I12" s="11" t="n"/>
       <c r="P12" s="11" t="n">
         <v>5458.48</v>
       </c>
-      <c r="W12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
-      <c r="AD12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
+      <c r="W12" s="11" t="n"/>
+      <c r="AD12" s="11" t="n"/>
       <c r="AF12" s="12">
         <f>SUM(B12:AE12)</f>
         <v/>
@@ -16053,21 +15481,13 @@
           <t>LB Hillingdon - Supported Living</t>
         </is>
       </c>
-      <c r="C13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
-      <c r="J13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
+      <c r="C13" s="11" t="n"/>
+      <c r="J13" s="11" t="n"/>
       <c r="Q13" s="11" t="n">
         <v>5203.8</v>
       </c>
-      <c r="X13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
-      <c r="AE13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
+      <c r="X13" s="11" t="n"/>
+      <c r="AE13" s="11" t="n"/>
       <c r="AF13" s="12">
         <f>SUM(B13:AE13)</f>
         <v/>
@@ -16079,18 +15499,12 @@
           <t>NHS Birmingham &amp; Solihull ICB</t>
         </is>
       </c>
-      <c r="D14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
-      <c r="K14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
+      <c r="D14" s="11" t="n"/>
+      <c r="K14" s="11" t="n"/>
       <c r="R14" s="11" t="n">
         <v>7814.17</v>
       </c>
-      <c r="Y14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
+      <c r="Y14" s="11" t="n"/>
       <c r="AF14" s="12">
         <f>SUM(B14:AE14)</f>
         <v/>
@@ -16102,18 +15516,12 @@
           <t>NHS Black Country ICB</t>
         </is>
       </c>
-      <c r="D15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
-      <c r="K15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
+      <c r="D15" s="11" t="n"/>
+      <c r="K15" s="11" t="n"/>
       <c r="R15" s="11" t="n">
         <v>5499.45</v>
       </c>
-      <c r="Y15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
+      <c r="Y15" s="11" t="n"/>
       <c r="AF15" s="12">
         <f>SUM(B15:AE15)</f>
         <v/>
@@ -16226,7 +15634,8 @@
           <t>Sandwell MBC - Supported Living</t>
         </is>
       </c>
-      <c r="H17" s="11" t="n">
+      <c r="H17" s="11" t="n"/>
+      <c r="O17" s="11" t="n">
         <v>132834.8</v>
       </c>
       <c r="AC17" s="11" t="n">
@@ -16243,18 +15652,12 @@
           <t>Solihull MBC - Supported Living</t>
         </is>
       </c>
-      <c r="G18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
-      <c r="N18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
+      <c r="G18" s="11" t="n"/>
+      <c r="N18" s="11" t="n"/>
       <c r="U18" s="11" t="n">
         <v>33031.6</v>
       </c>
-      <c r="AB18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
+      <c r="AB18" s="11" t="n"/>
       <c r="AF18" s="12">
         <f>SUM(B18:AE18)</f>
         <v/>
@@ -16266,21 +15669,13 @@
           <t>Walsall - Supported Living</t>
         </is>
       </c>
-      <c r="B19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
-      <c r="I19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
+      <c r="B19" s="11" t="n"/>
+      <c r="I19" s="11" t="n"/>
       <c r="P19" s="11" t="n">
         <v>319655.76</v>
       </c>
-      <c r="W19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
-      <c r="AD19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
+      <c r="W19" s="11" t="n"/>
+      <c r="AD19" s="11" t="n"/>
       <c r="AF19" s="12">
         <f>SUM(B19:AE19)</f>
         <v/>
@@ -16315,18 +15710,12 @@
           <t>People Plus - Direct Payments</t>
         </is>
       </c>
-      <c r="D21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
-      <c r="K21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
+      <c r="D21" s="11" t="n"/>
+      <c r="K21" s="11" t="n"/>
       <c r="R21" s="11" t="n">
         <v>21527.2</v>
       </c>
-      <c r="Y21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
+      <c r="Y21" s="11" t="n"/>
       <c r="AF21" s="12">
         <f>SUM(B21:AE21)</f>
         <v/>
@@ -16338,18 +15727,12 @@
           <t>Middlesbrough - Supported Living</t>
         </is>
       </c>
-      <c r="D22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
-      <c r="K22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
+      <c r="D22" s="11" t="n"/>
+      <c r="K22" s="11" t="n"/>
       <c r="R22" s="11" t="n">
         <v>6115.4</v>
       </c>
-      <c r="Y22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
+      <c r="Y22" s="11" t="n"/>
       <c r="AF22" s="12">
         <f>SUM(B22:AE22)</f>
         <v/>
@@ -17014,21 +16397,13 @@
           <t>Birmingham City Council - Supported Living</t>
         </is>
       </c>
-      <c r="B3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
-      <c r="I3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
+      <c r="B3" s="11" t="n"/>
+      <c r="I3" s="11" t="n"/>
       <c r="P3" s="11" t="n">
         <v>59419.08</v>
       </c>
-      <c r="W3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
-      <c r="AD3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
+      <c r="W3" s="11" t="n"/>
+      <c r="AD3" s="11" t="n"/>
       <c r="AG3" s="12">
         <f>SUM(B3:AF3)</f>
         <v/>
@@ -17074,6 +16449,9 @@
       <c r="Q6" s="11" t="n">
         <v>6585.35</v>
       </c>
+      <c r="AE6" s="11" t="n">
+        <v>6585.35</v>
+      </c>
       <c r="AG6" s="12">
         <f>SUM(B6:AF6)</f>
         <v/>
@@ -17122,18 +16500,12 @@
           <t>Walsall - Respite</t>
         </is>
       </c>
-      <c r="G9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
+      <c r="G9" s="11" t="n"/>
       <c r="N9" s="11" t="n">
         <v>11460.8</v>
       </c>
-      <c r="U9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
-      <c r="AB9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
+      <c r="U9" s="11" t="n"/>
+      <c r="AB9" s="11" t="n"/>
       <c r="AG9" s="12">
         <f>SUM(B9:AF9)</f>
         <v/>
@@ -17156,21 +16528,13 @@
           <t>Ideal for All Ltd - Direct Payments</t>
         </is>
       </c>
-      <c r="C11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
-      <c r="J11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
+      <c r="C11" s="11" t="n"/>
+      <c r="J11" s="11" t="n"/>
       <c r="Q11" s="11" t="n">
         <v>4131.62</v>
       </c>
-      <c r="X11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
-      <c r="AE11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
+      <c r="X11" s="11" t="n"/>
+      <c r="AE11" s="11" t="n"/>
       <c r="AG11" s="12">
         <f>SUM(B11:AF11)</f>
         <v/>
@@ -17182,18 +16546,12 @@
           <t>Kirklees - Supported Living</t>
         </is>
       </c>
-      <c r="G12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
+      <c r="G12" s="11" t="n"/>
       <c r="N12" s="11" t="n">
         <v>5458.48</v>
       </c>
-      <c r="U12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
-      <c r="AB12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
+      <c r="U12" s="11" t="n"/>
+      <c r="AB12" s="11" t="n"/>
       <c r="AG12" s="12">
         <f>SUM(B12:AF12)</f>
         <v/>
@@ -17205,18 +16563,12 @@
           <t>LB Hillingdon - Supported Living</t>
         </is>
       </c>
-      <c r="H13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
+      <c r="H13" s="11" t="n"/>
       <c r="O13" s="11" t="n">
         <v>5203.8</v>
       </c>
-      <c r="V13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
-      <c r="AC13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
+      <c r="V13" s="11" t="n"/>
+      <c r="AC13" s="11" t="n"/>
       <c r="AG13" s="12">
         <f>SUM(B13:AF13)</f>
         <v/>
@@ -17228,21 +16580,13 @@
           <t>NHS Birmingham &amp; Solihull ICB</t>
         </is>
       </c>
-      <c r="B14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
-      <c r="I14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
+      <c r="B14" s="11" t="n"/>
+      <c r="I14" s="11" t="n"/>
       <c r="P14" s="11" t="n">
         <v>7814.17</v>
       </c>
-      <c r="W14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
-      <c r="AD14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
+      <c r="W14" s="11" t="n"/>
+      <c r="AD14" s="11" t="n"/>
       <c r="AG14" s="12">
         <f>SUM(B14:AF14)</f>
         <v/>
@@ -17254,21 +16598,13 @@
           <t>NHS Black Country ICB</t>
         </is>
       </c>
-      <c r="B15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
-      <c r="I15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
+      <c r="B15" s="11" t="n"/>
+      <c r="I15" s="11" t="n"/>
       <c r="P15" s="11" t="n">
         <v>5499.45</v>
       </c>
-      <c r="W15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
-      <c r="AD15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
+      <c r="W15" s="11" t="n"/>
+      <c r="AD15" s="11" t="n"/>
       <c r="AG15" s="12">
         <f>SUM(B15:AF15)</f>
         <v/>
@@ -17384,7 +16720,8 @@
           <t>Sandwell MBC - Supported Living</t>
         </is>
       </c>
-      <c r="F17" s="11" t="n">
+      <c r="F17" s="11" t="n"/>
+      <c r="M17" s="11" t="n">
         <v>132834.8</v>
       </c>
       <c r="AA17" s="11" t="n">
@@ -17401,18 +16738,12 @@
           <t>Solihull MBC - Supported Living</t>
         </is>
       </c>
-      <c r="E18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
-      <c r="L18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
+      <c r="E18" s="11" t="n"/>
+      <c r="L18" s="11" t="n"/>
       <c r="S18" s="11" t="n">
         <v>33031.6</v>
       </c>
-      <c r="Z18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
+      <c r="Z18" s="11" t="n"/>
       <c r="AG18" s="12">
         <f>SUM(B18:AF18)</f>
         <v/>
@@ -17424,18 +16755,12 @@
           <t>Walsall - Supported Living</t>
         </is>
       </c>
-      <c r="G19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
+      <c r="G19" s="11" t="n"/>
       <c r="N19" s="11" t="n">
         <v>319655.76</v>
       </c>
-      <c r="U19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
-      <c r="AB19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
+      <c r="U19" s="11" t="n"/>
+      <c r="AB19" s="11" t="n"/>
       <c r="AG19" s="12">
         <f>SUM(B19:AF19)</f>
         <v/>
@@ -17473,21 +16798,13 @@
           <t>People Plus - Direct Payments</t>
         </is>
       </c>
-      <c r="B21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
-      <c r="I21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
+      <c r="B21" s="11" t="n"/>
+      <c r="I21" s="11" t="n"/>
       <c r="P21" s="11" t="n">
         <v>21527.2</v>
       </c>
-      <c r="W21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
-      <c r="AD21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
+      <c r="W21" s="11" t="n"/>
+      <c r="AD21" s="11" t="n"/>
       <c r="AG21" s="12">
         <f>SUM(B21:AF21)</f>
         <v/>
@@ -17499,21 +16816,13 @@
           <t>Middlesbrough - Supported Living</t>
         </is>
       </c>
-      <c r="B22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
-      <c r="I22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
+      <c r="B22" s="11" t="n"/>
+      <c r="I22" s="11" t="n"/>
       <c r="P22" s="11" t="n">
         <v>6115.4</v>
       </c>
-      <c r="W22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
-      <c r="AD22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
+      <c r="W22" s="11" t="n"/>
+      <c r="AD22" s="11" t="n"/>
       <c r="AG22" s="12">
         <f>SUM(B22:AF22)</f>
         <v/>

</xml_diff>

<commit_message>
Apply 4-weekly cadence to May 26 for consistency
May 26 rebuilt to the same literal cadence (total GBP1,806,573.78),
replacing the as-entered weekly-multiplied pattern.

https://claude.ai/code/session_01V6KrsFLkztukGdQb6oLmYN
</commit_message>
<xml_diff>
--- a/Income_forecast_2026.xlsx
+++ b/Income_forecast_2026.xlsx
@@ -10910,15 +10910,9 @@
           <t>Birmingham City Council - Supported Living</t>
         </is>
       </c>
-      <c r="H3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
-      <c r="O3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
-      <c r="V3" s="11" t="n">
-        <v>59419.08</v>
-      </c>
+      <c r="H3" s="11" t="n"/>
+      <c r="O3" s="11" t="n"/>
+      <c r="V3" s="11" t="n"/>
       <c r="AC3" s="11" t="n">
         <v>59419.08</v>
       </c>
@@ -11012,15 +11006,9 @@
           <t>Walsall - Respite</t>
         </is>
       </c>
-      <c r="F9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
-      <c r="M9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
-      <c r="T9" s="11" t="n">
-        <v>11460.8</v>
-      </c>
+      <c r="F9" s="11" t="n"/>
+      <c r="M9" s="11" t="n"/>
+      <c r="T9" s="11" t="n"/>
       <c r="AA9" s="11" t="n">
         <v>11460.8</v>
       </c>
@@ -11049,15 +11037,9 @@
       <c r="B11" s="11" t="n">
         <v>4131.62</v>
       </c>
-      <c r="I11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
-      <c r="P11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
-      <c r="W11" s="11" t="n">
-        <v>4131.62</v>
-      </c>
+      <c r="I11" s="11" t="n"/>
+      <c r="P11" s="11" t="n"/>
+      <c r="W11" s="11" t="n"/>
       <c r="AD11" s="11" t="n">
         <v>4131.62</v>
       </c>
@@ -11072,15 +11054,9 @@
           <t>Kirklees - Supported Living</t>
         </is>
       </c>
-      <c r="F12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
-      <c r="M12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
-      <c r="T12" s="11" t="n">
-        <v>5458.48</v>
-      </c>
+      <c r="F12" s="11" t="n"/>
+      <c r="M12" s="11" t="n"/>
+      <c r="T12" s="11" t="n"/>
       <c r="AA12" s="11" t="n">
         <v>5458.48</v>
       </c>
@@ -11095,15 +11071,9 @@
           <t>LB Hillingdon - Supported Living</t>
         </is>
       </c>
-      <c r="G13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
-      <c r="N13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
-      <c r="U13" s="11" t="n">
-        <v>5203.8</v>
-      </c>
+      <c r="G13" s="11" t="n"/>
+      <c r="N13" s="11" t="n"/>
+      <c r="U13" s="11" t="n"/>
       <c r="AB13" s="11" t="n">
         <v>5203.8</v>
       </c>
@@ -11118,15 +11088,9 @@
           <t>NHS Birmingham &amp; Solihull ICB</t>
         </is>
       </c>
-      <c r="H14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
-      <c r="O14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
-      <c r="V14" s="11" t="n">
-        <v>7814.17</v>
-      </c>
+      <c r="H14" s="11" t="n"/>
+      <c r="O14" s="11" t="n"/>
+      <c r="V14" s="11" t="n"/>
       <c r="AC14" s="11" t="n">
         <v>7814.17</v>
       </c>
@@ -11141,15 +11105,9 @@
           <t>NHS Black Country ICB</t>
         </is>
       </c>
-      <c r="H15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
-      <c r="O15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
-      <c r="V15" s="11" t="n">
-        <v>5499.45</v>
-      </c>
+      <c r="H15" s="11" t="n"/>
+      <c r="O15" s="11" t="n"/>
+      <c r="V15" s="11" t="n"/>
       <c r="AC15" s="11" t="n">
         <v>5499.45</v>
       </c>
@@ -11268,7 +11226,8 @@
           <t>Sandwell MBC - Supported Living</t>
         </is>
       </c>
-      <c r="E17" s="11" t="n">
+      <c r="E17" s="11" t="n"/>
+      <c r="L17" s="11" t="n">
         <v>132834.8</v>
       </c>
       <c r="Z17" s="11" t="n">
@@ -11288,15 +11247,9 @@
       <c r="D18" s="11" t="n">
         <v>33031.6</v>
       </c>
-      <c r="K18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
-      <c r="R18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
-      <c r="Y18" s="11" t="n">
-        <v>33031.6</v>
-      </c>
+      <c r="K18" s="11" t="n"/>
+      <c r="R18" s="11" t="n"/>
+      <c r="Y18" s="11" t="n"/>
       <c r="AF18" s="11" t="n">
         <v>33031.6</v>
       </c>
@@ -11311,15 +11264,9 @@
           <t>Walsall - Supported Living</t>
         </is>
       </c>
-      <c r="F19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
-      <c r="M19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
-      <c r="T19" s="11" t="n">
-        <v>319655.76</v>
-      </c>
+      <c r="F19" s="11" t="n"/>
+      <c r="M19" s="11" t="n"/>
+      <c r="T19" s="11" t="n"/>
       <c r="AA19" s="11" t="n">
         <v>319655.76</v>
       </c>
@@ -11357,15 +11304,9 @@
           <t>People Plus - Direct Payments</t>
         </is>
       </c>
-      <c r="H21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
-      <c r="O21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
-      <c r="V21" s="11" t="n">
-        <v>21527.2</v>
-      </c>
+      <c r="H21" s="11" t="n"/>
+      <c r="O21" s="11" t="n"/>
+      <c r="V21" s="11" t="n"/>
       <c r="AC21" s="11" t="n">
         <v>21527.2</v>
       </c>
@@ -11380,15 +11321,9 @@
           <t>Middlesbrough - Supported Living</t>
         </is>
       </c>
-      <c r="H22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
-      <c r="O22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
-      <c r="V22" s="11" t="n">
-        <v>6115.4</v>
-      </c>
+      <c r="H22" s="11" t="n"/>
+      <c r="O22" s="11" t="n"/>
+      <c r="V22" s="11" t="n"/>
       <c r="AC22" s="11" t="n">
         <v>6115.4</v>
       </c>

</xml_diff>